<commit_message>
Updated human deployment protocol and hardware testing spreadsheet
</commit_message>
<xml_diff>
--- a/TI_Workshop_HardwareTesting_Practical.xlsx
+++ b/TI_Workshop_HardwareTesting_Practical.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c9990f124d7388a/College/PhD/GLab/website/workshop material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12BFDC23-504C-49D6-83A3-88666169FF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{12BFDC23-504C-49D6-83A3-88666169FF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{255713F9-0513-46C1-8DFF-324E0E46226C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test info" sheetId="4" r:id="rId1"/>
@@ -370,9 +370,6 @@
     <t>Testing information</t>
   </si>
   <si>
-    <t>TI stSstimulator information</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -411,6 +408,9 @@
   </si>
   <si>
     <t>Use Oscilloscope.</t>
+  </si>
+  <si>
+    <t>TI Stimulator information</t>
   </si>
 </sst>
 </file>
@@ -565,10 +565,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -577,12 +581,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,6 +601,153 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>706277</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161990</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>308363</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>204760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3BD040A-E6E5-7B78-4CFE-6F1E44C6D8BF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="706277" y="1930919"/>
+          <a:ext cx="3204739" cy="2064402"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>772103</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>62095</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>316082</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>137103</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D111A0F6-21C9-7774-A8F3-76C797592619}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="772103" y="1829993"/>
+          <a:ext cx="3252956" cy="2095462"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>81643</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>322885</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>145105</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0BEC90C-2CD5-4F4A-92A9-4CAF5FA58C5E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="2113643"/>
+          <a:ext cx="3252956" cy="2095462"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
 <FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
   <bag type="Checkbox"/>
@@ -616,10 +763,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -959,13 +1102,13 @@
     </row>
     <row r="2" spans="2:3" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B2" s="14" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="2:3" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B3" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
@@ -990,17 +1133,17 @@
     </row>
     <row r="8" spans="2:3" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B8" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1032,18 +1175,18 @@
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="2:9" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="E2" s="15" t="s">
+      <c r="C2" s="16"/>
+      <c r="E2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="H2" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="15"/>
+      <c r="F2" s="16"/>
+      <c r="H2" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="16"/>
     </row>
     <row r="3" spans="2:9" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B3" s="2" t="s">
@@ -1060,14 +1203,14 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="15"/>
-      <c r="H4" s="15" t="s">
+      <c r="F4" s="16"/>
+      <c r="H4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="15"/>
+      <c r="I4" s="16"/>
     </row>
     <row r="5" spans="2:9" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B5" s="2" t="s">
@@ -1093,9 +1236,9 @@
     </row>
     <row r="7" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="19" t="b">
+        <v>58</v>
+      </c>
+      <c r="C7" s="15" t="b">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -1109,14 +1252,14 @@
       <c r="I7" s="4"/>
     </row>
     <row r="9" spans="2:9" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="H9" s="15" t="s">
+      <c r="F9" s="16"/>
+      <c r="H9" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="15"/>
+      <c r="I9" s="16"/>
     </row>
     <row r="10" spans="2:9" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="E10" s="13" t="s">
@@ -1341,6 +1484,7 @@
     <mergeCell ref="H4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>
@@ -1351,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EA9077D-ED0E-9348-9CA2-6CEB23EC113F}">
-  <dimension ref="B1:Q24"/>
+  <dimension ref="B1:Q26"/>
   <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -1378,10 +1522,10 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="2:17" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="16"/>
       <c r="E2" s="17" t="s">
         <v>3</v>
       </c>
@@ -1414,22 +1558,22 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
       <c r="J4" s="1"/>
-      <c r="L4" s="15" t="s">
+      <c r="L4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
     </row>
     <row r="5" spans="2:17" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B5" s="2" t="s">
@@ -1497,9 +1641,9 @@
     </row>
     <row r="7" spans="2:17" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="19" t="b">
+        <v>58</v>
+      </c>
+      <c r="C7" s="15" t="b">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -1639,80 +1783,80 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="6" t="s">
+    <row r="17" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" spans="2:17" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-    </row>
-    <row r="17" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
     </row>
     <row r="18" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="7" t="s">
-        <v>35</v>
-      </c>
+      <c r="B18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
     </row>
     <row r="19" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="10"/>
+      <c r="B19" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
     </row>
     <row r="20" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="10"/>
+      <c r="B20" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
     <row r="21" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="11" t="s">
-        <v>38</v>
+      <c r="B21" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
     </row>
     <row r="22" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="B22" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="10"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
     </row>
     <row r="23" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="7" t="s">
-        <v>43</v>
-      </c>
+      <c r="B23" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="10"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
     </row>
     <row r="24" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B24" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B25" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B26" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1725,12 +1869,13 @@
     <mergeCell ref="L4:Q4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F06CC8C-2D59-D94C-BC6D-4D39FCAF86C9}">
-  <dimension ref="B1:J24"/>
+  <dimension ref="B1:J27"/>
   <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -1753,16 +1898,16 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="2:10" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="E2" s="15" t="s">
+      <c r="C2" s="16"/>
+      <c r="E2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="3" spans="2:10" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B3" s="2" t="s">
@@ -1771,14 +1916,14 @@
       <c r="C3" s="2">
         <v>2</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16" t="s">
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="19"/>
     </row>
     <row r="4" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="2" t="s">
@@ -1810,7 +1955,7 @@
     </row>
     <row r="6" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" s="2">
         <v>6.8000000000000005E-2</v>
@@ -1830,30 +1975,30 @@
     </row>
     <row r="8" spans="2:10" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
     </row>
     <row r="9" spans="2:10" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16" t="s">
+      <c r="F9" s="19"/>
+      <c r="G9" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16" t="s">
+      <c r="H9" s="19"/>
+      <c r="I9" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="J9" s="16"/>
+      <c r="J9" s="19"/>
     </row>
     <row r="10" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E10" s="2" t="s">
@@ -1882,21 +2027,21 @@
         <v>26</v>
       </c>
       <c r="F12" s="5" t="e">
-        <f>(F10-F11)/(F10+F11)</f>
+        <f>(F10-ABS(F11))/(F10+ABS(F11))</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>26</v>
       </c>
       <c r="H12" s="5" t="e">
-        <f>(H10-H11)/(H10+H11)</f>
+        <f>(H10-ABS(H11))/(H10+ABS(H11))</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>26</v>
       </c>
       <c r="J12" s="5" t="e">
-        <f>(J10-J11)/(J10+J11)</f>
+        <f>(J10-ABS(J11))/(J10+ABS(J11))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -1911,75 +2056,77 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="6" t="s">
+    <row r="16" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="H16" s="8"/>
+    </row>
+    <row r="18" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-    </row>
-    <row r="16" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-    </row>
-    <row r="17" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="7" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+    </row>
+    <row r="20" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B20" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-    </row>
-    <row r="18" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="9" t="s">
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B21" s="9" t="s">
         <v>17</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="4"/>
-    </row>
-    <row r="20" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="4"/>
-    </row>
-    <row r="21" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="7" t="s">
+    <row r="22" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B22" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="10"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B23" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B24" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B25" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="12" t="s">
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B26" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="7" t="s">
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="2:7" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B27" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="4"/>
+      <c r="D27" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1993,5 +2140,6 @@
     <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>